<commit_message>
Napi adatok és HTML export frissítése
</commit_message>
<xml_diff>
--- a/data/hidegtarolas_export.xlsx
+++ b/data/hidegtarolas_export.xlsx
@@ -1,61 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arrivagroup-my.sharepoint.com/personal/sokvari_norbert_arrivabus_hu/Documents/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{20A3A44A-1C72-419D-A466-81D0CDE1E262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C513D8F-0E12-46F2-B3F4-099D6FA8A20D}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="4140" yWindow="18900" windowWidth="21600" windowHeight="11295" xr2:uid="{4AD81AF9-0199-4ABD-8C88-E50CAFDA8178}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4140" yWindow="18900" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Riport" sheetId="1" r:id="rId1"/>
+    <sheet name="Riport" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -70,22 +60,83 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -405,10 +456,572 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E3412-B789-441D-B168-440C0DF764A6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dátum</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Viszonylat</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Forda</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Rendszám</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Eredmény</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0960</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1340</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AAHY812</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>RENDBEN TÁROLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0710</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0710</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0710</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PDN623</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>RENDBEN TÁROLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1480</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AOJM873</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>AOGF659</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0350</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SGY804</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AOGF671</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AOGF672</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>RENDBEN TÁROLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AOIM014</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1821</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1840</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1480</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1820</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PDN609</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>RENDBEN TÁROLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0250</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2250</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AAHY805</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1821</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0360</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0360</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0360</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>ELTÉRÉS TÖRTÉNT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>